<commit_message>
Update MASTER Education Classes Roster.xlsx
</commit_message>
<xml_diff>
--- a/training/upload/MASTER Education Classes Roster.xlsx
+++ b/training/upload/MASTER Education Classes Roster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29819"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaronbell/Desktop/Git Repo Clone/CrewOps360/training/upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F33E49F-1EE7-4DD9-85D3-937C3435FD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{718697AD-6804-4364-B464-3C5139092EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17240" firstSheet="7" activeTab="7" xr2:uid="{5604E27C-0991-9B4E-A9D1-5F87A876A78F}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17240" firstSheet="8" activeTab="17" xr2:uid="{5604E27C-0991-9B4E-A9D1-5F87A876A78F}"/>
   </bookViews>
   <sheets>
     <sheet name="Class_Enrollment" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1343" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="269">
   <si>
     <t>STAFF NAME</t>
   </si>
@@ -12322,7 +12322,7 @@
         <v>191</v>
       </c>
       <c r="B7" s="6">
-        <v>46170</v>
+        <v>46142</v>
       </c>
       <c r="C7" s="12" t="b">
         <v>0</v>
@@ -12334,15 +12334,21 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" ht="15.75">
       <c r="A8" s="3" t="s">
         <v>192</v>
       </c>
+      <c r="B8" s="6">
+        <v>46170</v>
+      </c>
       <c r="C8" s="12" t="b">
         <v>0</v>
       </c>
       <c r="D8" s="12" t="b">
         <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -17724,7 +17730,7 @@
         <v>203</v>
       </c>
       <c r="B16" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -17816,20 +17822,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18016,11 +18022,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBE3643D-FDE0-44DC-9CDA-200C2597DFB6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13094262-B8A9-472E-A55D-BC65572C19CC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13094262-B8A9-472E-A55D-BC65572C19CC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBE3643D-FDE0-44DC-9CDA-200C2597DFB6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>